<commit_message>
Update proposal log to scope dashboard and show all table entries
Adjust proposal log to filter the dashboard by estimator initials for non-admins, always display all table entries, and refine the past-due bid display.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 44088ced-c7e0-44ac-8d9d-44e8eb10af50
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/K55ewxG
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-12.xlsx
+++ b/backups/proposal-log-2026-03-12.xlsx
@@ -49,15 +49,69 @@
     <t>Anticipated Finish</t>
   </si>
   <si>
-    <t>26-0018</t>
+    <t>26-0021</t>
+  </si>
+  <si>
+    <t>UCI 5000 Birch Dermatology</t>
+  </si>
+  <si>
+    <t>TM (LAX)</t>
+  </si>
+  <si>
+    <t>Special Projects</t>
+  </si>
+  <si>
+    <t>2026-03-05</t>
+  </si>
+  <si>
+    <t>2026-03-18</t>
+  </si>
+  <si>
+    <t>GT</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Estimating</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-11-30</t>
+  </si>
+  <si>
+    <t>26-0022</t>
+  </si>
+  <si>
+    <t>10900 Wilshire - High Rise - GMP for Award &amp; Mid-Rise Budget</t>
+  </si>
+  <si>
+    <t>2026-02-18</t>
+  </si>
+  <si>
+    <t>2026-03-16</t>
+  </si>
+  <si>
+    <t>GM</t>
+  </si>
+  <si>
+    <t>15000</t>
+  </si>
+  <si>
+    <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>2028-04-28</t>
+  </si>
+  <si>
+    <t>26-0023</t>
   </si>
   <si>
     <t>USC Keck Infill Building and Heart Hospital - Project F1</t>
   </si>
   <si>
-    <t>TM (LAX)</t>
-  </si>
-  <si>
     <t>Healthcare</t>
   </si>
   <si>
@@ -67,67 +121,13 @@
     <t>2026-03-11</t>
   </si>
   <si>
-    <t>HK</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>Estimating</t>
+    <t>20000</t>
   </si>
   <si>
     <t>2026-03-17</t>
   </si>
   <si>
     <t>2027-11-29</t>
-  </si>
-  <si>
-    <t>26-0019</t>
-  </si>
-  <si>
-    <t>10900 Wilshire - High Rise - GMP for Award &amp; Mid-Rise Budget</t>
-  </si>
-  <si>
-    <t>Special Projects</t>
-  </si>
-  <si>
-    <t>2026-02-18</t>
-  </si>
-  <si>
-    <t>2026-03-16</t>
-  </si>
-  <si>
-    <t>GT</t>
-  </si>
-  <si>
-    <t>2026-05-01</t>
-  </si>
-  <si>
-    <t>2028-04-28</t>
-  </si>
-  <si>
-    <t>26-0020</t>
-  </si>
-  <si>
-    <t>UCI 5000 Birch Dermatology</t>
-  </si>
-  <si>
-    <t>2026-03-05</t>
-  </si>
-  <si>
-    <t>2026-03-18</t>
-  </si>
-  <si>
-    <t>GM</t>
-  </si>
-  <si>
-    <t>2026-04-01</t>
-  </si>
-  <si>
-    <t>2026-11-30</t>
   </si>
 </sst>
 </file>
@@ -604,68 +604,68 @@
         <v>19</v>
       </c>
       <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
         <v>20</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>22</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
         <v>24</v>
-      </c>
-      <c r="B3" t="s">
-        <v>25</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
         <v>26</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>27</v>
-      </c>
-      <c r="F3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" t="s">
-        <v>29</v>
       </c>
       <c r="H3" t="s">
         <v>19</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="J3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" t="s">
         <v>30</v>
-      </c>
-      <c r="L3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
         <v>32</v>
-      </c>
-      <c r="B4" t="s">
-        <v>33</v>
       </c>
       <c r="C4" t="s">
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
         <v>34</v>
@@ -674,16 +674,16 @@
         <v>35</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="H4" t="s">
         <v>19</v>
       </c>
       <c r="I4" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="J4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K4" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Show all project proposals in the user's dashboard view
Modify the `getDashFiltered` function to include unassigned proposals in the dashboard view for all users.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0e3e820c-8a96-4736-8cca-5cbd8e47380c
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/K55ewxG
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-03-12.xlsx
+++ b/backups/proposal-log-2026-03-12.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -49,79 +49,28 @@
     <t>Anticipated Finish</t>
   </si>
   <si>
-    <t>26-0021</t>
-  </si>
-  <si>
-    <t>UCI 5000 Birch Dermatology</t>
+    <t>26-0024</t>
+  </si>
+  <si>
+    <t>USC Keck Infill Building and Heart Hospital - Project F1</t>
   </si>
   <si>
     <t>TM (LAX)</t>
   </si>
   <si>
-    <t>Special Projects</t>
-  </si>
-  <si>
-    <t>2026-03-05</t>
-  </si>
-  <si>
-    <t>2026-03-18</t>
-  </si>
-  <si>
-    <t>GT</t>
+    <t>Healthcare</t>
+  </si>
+  <si>
+    <t>2026-03-04</t>
+  </si>
+  <si>
+    <t>2026-03-11</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
     <t>Estimating</t>
-  </si>
-  <si>
-    <t>2026-04-01</t>
-  </si>
-  <si>
-    <t>2026-11-30</t>
-  </si>
-  <si>
-    <t>26-0022</t>
-  </si>
-  <si>
-    <t>10900 Wilshire - High Rise - GMP for Award &amp; Mid-Rise Budget</t>
-  </si>
-  <si>
-    <t>2026-02-18</t>
-  </si>
-  <si>
-    <t>2026-03-16</t>
-  </si>
-  <si>
-    <t>GM</t>
-  </si>
-  <si>
-    <t>15000</t>
-  </si>
-  <si>
-    <t>2026-05-01</t>
-  </si>
-  <si>
-    <t>2028-04-28</t>
-  </si>
-  <si>
-    <t>26-0023</t>
-  </si>
-  <si>
-    <t>USC Keck Infill Building and Heart Hospital - Project F1</t>
-  </si>
-  <si>
-    <t>Healthcare</t>
-  </si>
-  <si>
-    <t>2026-03-04</t>
-  </si>
-  <si>
-    <t>2026-03-11</t>
-  </si>
-  <si>
-    <t>20000</t>
   </si>
   <si>
     <t>2026-03-17</t>
@@ -526,7 +475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -601,99 +550,23 @@
         <v>18</v>
       </c>
       <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>20</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>21</v>
-      </c>
-      <c r="L2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" t="s">
-        <v>29</v>
-      </c>
-      <c r="L3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" t="s">
-        <v>35</v>
-      </c>
-      <c r="G4" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" t="s">
-        <v>37</v>
-      </c>
-      <c r="L4" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L4"/>
+  <autoFilter ref="A1:L2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>